<commit_message>
feat: enhance voter import functionality with date formatting and improved password generation
</commit_message>
<xml_diff>
--- a/server/imports/voters.xlsx
+++ b/server/imports/voters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RAWJET\github\E-Election\server\imports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AF070D-6F35-49CA-AF69-310F73F58226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4850FD9-1BA0-4DE1-8696-9D56C000712B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="D4" s="1">
-        <v>40497</v>
+        <v>39036</v>
       </c>
       <c r="E4" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
feat: update navigation items in PortalShell; remove deprecated 'System Settings' link
</commit_message>
<xml_diff>
--- a/server/imports/voters.xlsx
+++ b/server/imports/voters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RAWJET\github\E-Election\server\imports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4850FD9-1BA0-4DE1-8696-9D56C000712B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD9973F-CE01-43BB-9DE4-84C705C93695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
   <si>
     <t>EPIC Number</t>
   </si>
@@ -101,9 +101,6 @@
     <t>Amritsar</t>
   </si>
   <si>
-    <t>Ward 6</t>
-  </si>
-  <si>
     <t>Green Avenue</t>
   </si>
   <si>
@@ -137,9 +134,6 @@
     <t>9227745839</t>
   </si>
   <si>
-    <t>Ward 9</t>
-  </si>
-  <si>
     <t>GT Road</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
     <t>9603076873</t>
   </si>
   <si>
-    <t>Ward 4</t>
-  </si>
-  <si>
     <t>Queens Road</t>
   </si>
   <si>
@@ -186,6 +177,9 @@
   </si>
   <si>
     <t>Fatehgarh Churian</t>
+  </si>
+  <si>
+    <t>Ward 25</t>
   </si>
 </sst>
 </file>
@@ -592,16 +586,16 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D2" s="1">
         <v>38518</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
         <v>19</v>
@@ -616,10 +610,10 @@
         <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="K2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L2" t="s">
         <v>21</v>
@@ -628,24 +622,24 @@
         <v>13</v>
       </c>
       <c r="N2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O2">
         <v>143003</v>
       </c>
       <c r="P2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" t="s">
         <v>24</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
@@ -654,10 +648,10 @@
         <v>37506</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
         <v>20</v>
@@ -669,10 +663,10 @@
         <v>21</v>
       </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L3" t="s">
         <v>21</v>
@@ -681,24 +675,24 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O3">
         <v>143007</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -707,10 +701,10 @@
         <v>39036</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -722,10 +716,10 @@
         <v>21</v>
       </c>
       <c r="J4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="K4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L4" t="s">
         <v>21</v>
@@ -734,36 +728,36 @@
         <v>29</v>
       </c>
       <c r="N4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O4">
         <v>143001</v>
       </c>
       <c r="P4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Q4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="1">
         <v>27121</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -775,10 +769,10 @@
         <v>21</v>
       </c>
       <c r="J5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" t="s">
         <v>39</v>
-      </c>
-      <c r="K5" t="s">
-        <v>42</v>
       </c>
       <c r="L5" t="s">
         <v>21</v>
@@ -787,16 +781,16 @@
         <v>82</v>
       </c>
       <c r="N5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O5">
         <v>143009</v>
       </c>
       <c r="P5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="Q5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">

</xml_diff>